<commit_message>
Market-implied model: apply the synthesis audit (event-sd input, lognormal probabilities, retired guide numbers, drifted figures)
Synthesis audit passed with fixes, no blockers (research/notes/reverse_dcf/audit_synthesis.md). Applied: parse the
options event sd from B's text field (was blank in the workbook); use the lognormal 12-month P(above) throughout
(was the skew-adjusted series against a lognormal caption); replace the two retired 4Q26 guide numbers in the print
scenarios with C's post-repair values ($3,102m, $3,121m); correct eleven figures in the note to their CSV sources;
tighten the run synthesis wording. Recon unchanged at 0.0014.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WRusgUtfi8DDbuqa6opoBR
</commit_message>
<xml_diff>
--- a/model/ABNB_market_implied.xlsx
+++ b/model/ABNB_market_implied.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krish\citadel-abnb-reversedcf\model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{954255F7-D536-4B18-8A01-42BDE8E73F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92AAE067-391E-4DC8-BC7D-3F69EE1E4445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -331,7 +331,7 @@
     <t>Fixed 16.5x: nights (%)</t>
   </si>
   <si>
-    <t>P(price above this in 12M, options RN)</t>
+    <t>P(price above this in 12M, options RN, lognormal)</t>
   </si>
   <si>
     <t>P(above at 20 Nov, options RN)</t>
@@ -403,7 +403,7 @@
     <t>Implied FY27 nights growth (%)</t>
   </si>
   <si>
-    <t>P(above joint-solve price in 12M, options RN)</t>
+    <t>P(above joint-solve price in 12M, options RN, lognormal)</t>
   </si>
   <si>
     <t>Management literal</t>
@@ -469,7 +469,7 @@
     <t>Team base (WS29/30)</t>
   </si>
   <si>
-    <t>Team base, ex-NA lap adopted</t>
+    <t>Team base, ex-NA lap adopted (4Q26 8.1%, team elasticity)</t>
   </si>
   <si>
     <t>Q3 nowcast central (reviews index), 4Q26 at team revenue</t>
@@ -1630,13 +1630,13 @@
     <t>Team base (WS29/30):E_S2_post2022</t>
   </si>
   <si>
-    <t>Team base, ex-NA lap adopted:E_S2_ex_reopening</t>
-  </si>
-  <si>
-    <t>Team base, ex-NA lap adopted:E_S1_post2022</t>
-  </si>
-  <si>
-    <t>Team base, ex-NA lap adopted:E_S2_post2022</t>
+    <t>Team base, ex-NA lap adopted (4Q26 8.1%, team elasticity):E_S2_ex_reopening</t>
+  </si>
+  <si>
+    <t>Team base, ex-NA lap adopted (4Q26 8.1%, team elasticity):E_S1_post2022</t>
+  </si>
+  <si>
+    <t>Team base, ex-NA lap adopted (4Q26 8.1%, team elasticity):E_S2_post2022</t>
   </si>
   <si>
     <t>Q3 nowcast central (reviews index), 4Q26 at team revenue:E_S2_ex_reopening</t>
@@ -2531,7 +2531,9 @@
       <c r="A35" t="s">
         <v>72</v>
       </c>
-      <c r="B35" s="4"/>
+      <c r="B35" s="4">
+        <v>9.5</v>
+      </c>
       <c r="C35" s="5" t="s">
         <v>73</v>
       </c>
@@ -2540,7 +2542,9 @@
       <c r="A36" t="s">
         <v>74</v>
       </c>
-      <c r="B36" s="4"/>
+      <c r="B36" s="4">
+        <v>7.6</v>
+      </c>
       <c r="C36" s="5" t="s">
         <v>75</v>
       </c>
@@ -2708,7 +2712,7 @@
         <v>-24.931939934577898</v>
       </c>
       <c r="S5" s="10">
-        <v>0.74099999999999999</v>
+        <v>0.75</v>
       </c>
       <c r="T5" s="10">
         <v>0.95099999999999996</v>
@@ -2786,7 +2790,7 @@
         <v>-8.1253491301772396</v>
       </c>
       <c r="S6" s="10">
-        <v>0.59899999999999998</v>
+        <v>0.58799999999999997</v>
       </c>
       <c r="T6" s="10">
         <v>0.75</v>
@@ -2868,7 +2872,7 @@
         <v>1.3412203841382198</v>
       </c>
       <c r="S7" s="10">
-        <v>0.51700000000000002</v>
+        <v>0.5</v>
       </c>
       <c r="T7" s="10">
         <v>0.58199999999999996</v>
@@ -2946,7 +2950,7 @@
         <v>2.164400341904793</v>
       </c>
       <c r="S8" s="10">
-        <v>0.51</v>
+        <v>0.49299999999999999</v>
       </c>
       <c r="T8" s="10">
         <v>0.56499999999999995</v>
@@ -3028,7 +3032,7 @@
         <v>5.7246536592451491</v>
       </c>
       <c r="S9" s="10">
-        <v>0.48</v>
+        <v>0.46200000000000002</v>
       </c>
       <c r="T9" s="10">
         <v>0.49299999999999999</v>
@@ -3110,7 +3114,7 @@
         <v>12.111158164917413</v>
       </c>
       <c r="S10" s="10">
-        <v>0.42799999999999999</v>
+        <v>0.40899999999999997</v>
       </c>
       <c r="T10" s="10">
         <v>0.36599999999999999</v>
@@ -3192,7 +3196,7 @@
         <v>15.884066304680843</v>
       </c>
       <c r="S11" s="10">
-        <v>0.39900000000000002</v>
+        <v>0.379</v>
       </c>
       <c r="T11" s="10">
         <v>0.29699999999999999</v>
@@ -3274,7 +3278,7 @@
         <v>24.458857531415855</v>
       </c>
       <c r="S12" s="10">
-        <v>0.33600000000000002</v>
+        <v>0.318</v>
       </c>
       <c r="T12" s="10">
         <v>0.17</v>
@@ -3356,7 +3360,7 @@
         <v>35.708983620892184</v>
       </c>
       <c r="S13" s="10">
-        <v>0.26300000000000001</v>
+        <v>0.25</v>
       </c>
       <c r="T13" s="10">
         <v>6.9000000000000006E-2</v>
@@ -3434,7 +3438,7 @@
         <v>39.893481739538906</v>
       </c>
       <c r="S14" s="10">
-        <v>0.23899999999999999</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="T14" s="10">
         <v>4.7E-2</v>
@@ -3530,7 +3534,7 @@
         <v>7.2757906663280636</v>
       </c>
       <c r="I5" s="10">
-        <v>0.52700000000000002</v>
+        <v>0.51</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -3564,7 +3568,7 @@
         <v>9.9823211111328192</v>
       </c>
       <c r="I6" s="10">
-        <v>0.45</v>
+        <v>0.432</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -3598,7 +3602,7 @@
         <v>15.238811509835703</v>
       </c>
       <c r="I7" s="10">
-        <v>0.313</v>
+        <v>0.29699999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -3632,7 +3636,7 @@
         <v>8.0623547107889983</v>
       </c>
       <c r="I8" s="10">
-        <v>0.504</v>
+        <v>0.48699999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -3666,7 +3670,7 @@
         <v>8.4651598913871418</v>
       </c>
       <c r="I9" s="10">
-        <v>0.49299999999999999</v>
+        <v>0.47499999999999998</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -3700,7 +3704,7 @@
         <v>-1.729307886151854</v>
       </c>
       <c r="I10" s="10">
-        <v>0.75</v>
+        <v>0.76100000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -3734,7 +3738,7 @@
         <v>16.056435701588168</v>
       </c>
       <c r="I11" s="10">
-        <v>0.29299999999999998</v>
+        <v>0.27800000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -3828,7 +3832,7 @@
       </c>
       <c r="I5" s="7">
         <f>Inputs!$B$35</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="J5" s="7">
         <f>-(Inputs!$B$30+Inputs!$B$31*C5)/Inputs!$B$32</f>
@@ -3851,15 +3855,15 @@
         <v>-1</v>
       </c>
       <c r="D6" s="12">
-        <v>3055</v>
+        <v>3102</v>
       </c>
       <c r="E6" s="7">
         <f>(D6/Inputs!$B$27-1)*100</f>
-        <v>-3.1388712745719749</v>
+        <v>-1.6487000634115456</v>
       </c>
       <c r="F6" s="7">
         <f>Inputs!$B$30+Inputs!$B$31*C6+Inputs!$B$32*E6</f>
-        <v>-12.189819277108439</v>
+        <v>-9.1206626506024193</v>
       </c>
       <c r="G6" s="7">
         <f>Inputs!$B$33+Inputs!$B$34*C6</f>
@@ -3867,11 +3871,11 @@
       </c>
       <c r="H6" s="7">
         <f t="shared" si="0"/>
-        <v>-10.578957260621436</v>
+        <v>-8.6082058338617689</v>
       </c>
       <c r="I6" s="7">
         <f>Inputs!$B$35</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="J6" s="7">
         <f>-(Inputs!$B$30+Inputs!$B$31*C6)/Inputs!$B$32</f>
@@ -3894,15 +3898,15 @@
         <v>-1</v>
       </c>
       <c r="D7" s="12">
-        <v>3107</v>
+        <v>3121</v>
       </c>
       <c r="E7" s="7">
         <f>(D7/Inputs!$B$27-1)*100</f>
-        <v>-1.4901712111604293</v>
+        <v>-1.0462904248573213</v>
       </c>
       <c r="F7" s="7">
         <f>Inputs!$B$30+Inputs!$B$31*C7+Inputs!$B$32*E7</f>
-        <v>-8.7941566265060196</v>
+        <v>-7.8799397590361391</v>
       </c>
       <c r="G7" s="7">
         <f>Inputs!$B$33+Inputs!$B$34*C7</f>
@@ -3910,11 +3914,11 @@
       </c>
       <c r="H7" s="7">
         <f t="shared" si="0"/>
-        <v>-8.398551426759667</v>
+        <v>-7.8115190868738065</v>
       </c>
       <c r="I7" s="7">
         <f>Inputs!$B$35</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="J7" s="7">
         <f>-(Inputs!$B$30+Inputs!$B$31*C7)/Inputs!$B$32</f>
@@ -3957,7 +3961,7 @@
       </c>
       <c r="I8" s="7">
         <f>Inputs!$B$35</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="J8" s="7">
         <f>-(Inputs!$B$30+Inputs!$B$31*C8)/Inputs!$B$32</f>
@@ -4000,7 +4004,7 @@
       </c>
       <c r="I9" s="7">
         <f>Inputs!$B$35</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="J9" s="7">
         <f>-(Inputs!$B$30+Inputs!$B$31*C9)/Inputs!$B$32</f>
@@ -4043,7 +4047,7 @@
       </c>
       <c r="I10" s="7">
         <f>Inputs!$B$35</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="J10" s="7">
         <f>-(Inputs!$B$30+Inputs!$B$31*C10)/Inputs!$B$32</f>
@@ -4086,7 +4090,7 @@
       </c>
       <c r="I11" s="7">
         <f>Inputs!$B$35</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="J11" s="7">
         <f>-(Inputs!$B$30+Inputs!$B$31*C11)/Inputs!$B$32</f>
@@ -4129,7 +4133,7 @@
       </c>
       <c r="I12" s="7">
         <f>Inputs!$B$35</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="J12" s="7">
         <f>-(Inputs!$B$30+Inputs!$B$31*C12)/Inputs!$B$32</f>
@@ -4172,7 +4176,7 @@
       </c>
       <c r="I13" s="7">
         <f>Inputs!$B$35</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="J13" s="7">
         <f>-(Inputs!$B$30+Inputs!$B$31*C13)/Inputs!$B$32</f>
@@ -7242,7 +7246,7 @@
       </c>
       <c r="H4" s="9">
         <f>Market_Implied!S9</f>
-        <v>0.48</v>
+        <v>0.46200000000000002</v>
       </c>
       <c r="I4" s="7"/>
       <c r="J4" t="s">
@@ -7279,7 +7283,7 @@
       </c>
       <c r="H5" s="9">
         <f>Market_Implied!S9</f>
-        <v>0.48</v>
+        <v>0.46200000000000002</v>
       </c>
       <c r="I5" s="7"/>
       <c r="J5" t="s">
@@ -7316,7 +7320,7 @@
       </c>
       <c r="H6" s="9">
         <f>Market_Implied!S9</f>
-        <v>0.48</v>
+        <v>0.46200000000000002</v>
       </c>
       <c r="I6" s="7"/>
       <c r="J6" t="s">
@@ -7353,7 +7357,7 @@
       </c>
       <c r="H7" s="9">
         <f>Market_Implied!S5</f>
-        <v>0.74099999999999999</v>
+        <v>0.75</v>
       </c>
       <c r="I7" s="7"/>
       <c r="J7" t="s">
@@ -7390,7 +7394,7 @@
       </c>
       <c r="H8" s="9">
         <f>Market_Implied!S7</f>
-        <v>0.51700000000000002</v>
+        <v>0.5</v>
       </c>
       <c r="I8" s="7"/>
       <c r="J8" t="s">
@@ -7427,7 +7431,7 @@
       </c>
       <c r="H9" s="9">
         <f>Market_Implied!S13</f>
-        <v>0.26300000000000001</v>
+        <v>0.25</v>
       </c>
       <c r="I9" s="7"/>
       <c r="J9" t="s">
@@ -7464,7 +7468,7 @@
       </c>
       <c r="H10" s="9">
         <f>Market_Implied!S8</f>
-        <v>0.51</v>
+        <v>0.49299999999999999</v>
       </c>
       <c r="I10" s="7"/>
       <c r="J10" t="s">
@@ -7501,7 +7505,7 @@
       </c>
       <c r="H11" s="9">
         <f>Market_Implied!S10</f>
-        <v>0.42799999999999999</v>
+        <v>0.40899999999999997</v>
       </c>
       <c r="I11" s="7"/>
       <c r="J11" t="s">
@@ -7538,7 +7542,7 @@
       </c>
       <c r="H12" s="9">
         <f>Market_Implied!S12</f>
-        <v>0.33600000000000002</v>
+        <v>0.318</v>
       </c>
       <c r="I12" s="7"/>
       <c r="J12" t="s">
@@ -7575,7 +7579,7 @@
       </c>
       <c r="H13" s="9">
         <f>Market_Implied!S14</f>
-        <v>0.23899999999999999</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="I13" s="7"/>
       <c r="J13" t="s">
@@ -7612,7 +7616,7 @@
       </c>
       <c r="H14" s="9">
         <f>Cases!I5</f>
-        <v>0.52700000000000002</v>
+        <v>0.51</v>
       </c>
       <c r="I14" s="7"/>
       <c r="J14" t="s">
@@ -7649,7 +7653,7 @@
       </c>
       <c r="H15" s="9">
         <f>Cases!I6</f>
-        <v>0.45</v>
+        <v>0.432</v>
       </c>
       <c r="I15" s="7">
         <f>Print_5Nov!G9</f>
@@ -7689,7 +7693,7 @@
       </c>
       <c r="H16" s="9">
         <f>Cases!I7</f>
-        <v>0.313</v>
+        <v>0.29699999999999999</v>
       </c>
       <c r="I16" s="7"/>
       <c r="J16" t="s">
@@ -7726,7 +7730,7 @@
       </c>
       <c r="H17" s="9">
         <f>Cases!I8</f>
-        <v>0.504</v>
+        <v>0.48699999999999999</v>
       </c>
       <c r="I17" s="7">
         <f>Print_5Nov!G8</f>
@@ -7766,7 +7770,7 @@
       </c>
       <c r="H18" s="9">
         <f>Cases!I9</f>
-        <v>0.49299999999999999</v>
+        <v>0.47499999999999998</v>
       </c>
       <c r="I18" s="7">
         <f>Print_5Nov!G5</f>
@@ -7806,7 +7810,7 @@
       </c>
       <c r="H19" s="9">
         <f>Cases!I10</f>
-        <v>0.75</v>
+        <v>0.76100000000000001</v>
       </c>
       <c r="I19" s="7"/>
       <c r="J19" t="s">
@@ -7843,7 +7847,7 @@
       </c>
       <c r="H20" s="9">
         <f>Cases!I11</f>
-        <v>0.29299999999999998</v>
+        <v>0.27800000000000002</v>
       </c>
       <c r="I20" s="7"/>
       <c r="J20" t="s">
@@ -10460,10 +10464,10 @@
         <v>529</v>
       </c>
       <c r="C155">
-        <v>-12.189819277108439</v>
+        <v>-9.1206626506024193</v>
       </c>
       <c r="D155">
-        <v>-12.189819277108439</v>
+        <v>-9.1206626506024193</v>
       </c>
       <c r="E155">
         <v>0</v>
@@ -10494,10 +10498,10 @@
         <v>531</v>
       </c>
       <c r="C157">
-        <v>-10.57895726062144</v>
+        <v>-8.6082058338617689</v>
       </c>
       <c r="D157">
-        <v>-10.57895726062144</v>
+        <v>-8.6082058338617689</v>
       </c>
       <c r="E157">
         <v>0</v>
@@ -10511,10 +10515,10 @@
         <v>532</v>
       </c>
       <c r="C158">
-        <v>-8.7941566265060196</v>
+        <v>-7.8799397590361391</v>
       </c>
       <c r="D158">
-        <v>-8.7941566265060196</v>
+        <v>-7.8799397590361391</v>
       </c>
       <c r="E158">
         <v>0</v>
@@ -10545,10 +10549,10 @@
         <v>534</v>
       </c>
       <c r="C160">
-        <v>-8.398551426759667</v>
+        <v>-7.8115190868738056</v>
       </c>
       <c r="D160">
-        <v>-8.398551426759667</v>
+        <v>-7.8115190868738056</v>
       </c>
       <c r="E160">
         <v>0</v>

</xml_diff>